<commit_message>
RoadPro 3.0: guide, shortcuts and page content
- Guide (PDF 19 pages, PowerPoint) and shortcut sheet replaced with 3.0.
- New commands on the page: RDJ (junction / tie-in with kerb returns)
  and RDM (road markings); RDW/RDT note that each side can have its own
  chainages and radius; chainage input 100 or 0+100.
- 'New in RoadPro 3.0' box after the hero; ROAD-JUNCTION layer; report
  rows for junction setting-out and road markings; three new quick fixes.
- 'Look inside the user guide': eight 3.0 pages, including the new
  junction and road markings pages, from a new guide-v3 folder.
- Home spotlight mentions junctions and road markings.

The plugin download (RoadPro.zip) is still 2.6 until the 3.0 RoadPro.lsp
is added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBEY1H8rXcGm4de5BZo5nb
</commit_message>
<xml_diff>
--- a/public/roadpro/RoadPro_Shortcuts.xlsx
+++ b/public/roadpro/RoadPro_Shortcuts.xlsx
@@ -183,9 +183,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -551,25 +549,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RoadPro v2.6 - Shortcut Keys</t>
+          <t>RoadPro v3.0 - Shortcut Keys</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AutoCAD road builder plugin  |  05-Oct-2026  |  Developed by https://www.exceltokml.com/</t>
+          <t>AutoCAD road builder plugin  |  07-Oct-2026  |  Developed by https://www.exceltokml.com/</t>
         </is>
       </c>
     </row>
@@ -682,7 +680,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>RDW</t>
@@ -695,11 +693,11 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Lane widening: extra lane from start to end chainage that comes back, straight or curve taper, fillet or direct link</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
+          <t>Lane widening: extra lane from start to end chainage that comes back, straight or curve taper, fillet or direct link. Both sides can use different chainages and radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>RDT</t>
@@ -712,69 +710,77 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Road taper: wider (+) or narrower (-) from any start to any end chainage, new width continues to the road end</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
+          <t>Road taper: wider (+) or narrower (-) from any start to any end chainage, new width continues to the road end. Both sides can use different chainages and radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
+          <t>RDJ</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>ROADJUNCTION</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Road junction / tie-in: join a new road with kerb-return radius, opened edge, corner surface, barricades, STOP / GIVE WAY and turning-area markings</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>RDM</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>ROADMARK</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Road markings: white edge lines and lane line (broken 3 m / 6 m, solid on bends and junction approaches). Draw again to refresh, or Remove</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>ROADPRORESET</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Restore all settings to defaults (no shortcut, on purpose, so you don't reset by accident)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Useful AutoCAD keys while using RoadPro</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Use</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Undo the whole road in one step</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Open the command history to see the summary and the Excel file path</t>
         </is>
       </c>
       <c r="C18" s="11" t="n"/>
@@ -782,12 +788,12 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Enter</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Finish drawing the centre line, or skip a prompt (such as placing tables)</t>
+          <t>Undo the whole road in one step</t>
         </is>
       </c>
       <c r="C19" s="11" t="n"/>
@@ -795,12 +801,12 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Esc</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Cancel the command</t>
+          <t>Open the command history to see the summary and the Excel file path</t>
         </is>
       </c>
       <c r="C20" s="11" t="n"/>
@@ -808,25 +814,51 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Enter</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Finish drawing the centre line, or skip a prompt (such as placing tables)</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Esc</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Cancel the command</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>APPLOAD</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Load RoadPro.lsp, or add it to the Startup Suite</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Note: RDR, RDRAD, RDSEC, RDX, RDW and RDT all start by asking you to select the road's centre line (layer ROAD-CL). Turning radius is measured at the centre line by default.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="C23" s="11" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Note: RDR, RDRAD, RDSEC, RDX, RDW, RDT, RDJ and RDM all start by asking you to select the road's centre line (layer ROAD-CL). Turning radius is measured at the centre line by default. Chainage boxes accept 100 or 0+100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Developed by https://www.exceltokml.com/</t>
         </is>
@@ -836,25 +868,25 @@
   <mergeCells count="12">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B16:C16"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;9 RoadPro v2.6  |  Developed by https://www.exceltokml.com/</oddFooter>
+    <oddFooter>&amp;C&amp;9 RoadPro v3.0  |  Developed by https://www.exceltokml.com/</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
RoadPro 3.2: auxiliary lane and island, standard signs and markings, 22-page guide
New plugin zip (RoadPro.lsp 3.2 with README), user guide PDF/PPTX and
shortcut sheet; guide previews re-rendered into guide-v32; What's new,
commands, defaults, report and fixes updated; standards note added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBEY1H8rXcGm4de5BZo5nb
</commit_message>
<xml_diff>
--- a/public/roadpro/RoadPro_Shortcuts.xlsx
+++ b/public/roadpro/RoadPro_Shortcuts.xlsx
@@ -560,14 +560,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RoadPro v3.0 - Shortcut Keys</t>
+          <t>RoadPro v3.2 - Shortcut Keys</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AutoCAD road builder plugin  |  07-Oct-2026  |  Developed by https://www.exceltokml.com/</t>
+          <t>AutoCAD road builder plugin  |  09-Oct-2026  |  Developed by https://www.exceltokml.com/</t>
         </is>
       </c>
     </row>
@@ -850,10 +850,10 @@
       </c>
       <c r="C23" s="11" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="44" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Note: RDR, RDRAD, RDSEC, RDX, RDW, RDT, RDJ and RDM all start by asking you to select the road's centre line (layer ROAD-CL). Turning radius is measured at the centre line by default. Chainage boxes accept 100 or 0+100.</t>
+          <t>Note: RDR, RDRAD, RDSEC, RDX, RDW, RDT, RDJ and RDM all start by asking you to select the road's centre line (layer ROAD-CL). Turning radius: Match existing (default) or Manual, measured at the centre line. Chainage boxes accept 100 or 0+100. Sign sizes, warning distances and line patterns follow Oman HDS 2017 Sec.19 (check QTCM in Qatar).</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;9 RoadPro v3.0  |  Developed by https://www.exceltokml.com/</oddFooter>
+    <oddFooter>&amp;C&amp;9 RoadPro v3.2  |  Developed by https://www.exceltokml.com/</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
RoadPro 3.3: single line (RDL), junction corners, cones and kerb follow widening
- The plugin, user guide (PDF and PowerPoint, now 38 pages) and shortcut
  sheet replaced with 3.3. RoadPro.zip holds RoadPro.lsp and the new README.
- /roadpro: new in 3.3 (RDL single line of barricades, cones or kerb on any
  line; RDJ corner treatment; cones and kerb follow RDW / RDT; kerb units and
  cone band), an upgrade note from 3.2, RDL in the command table, new
  defaults, layers, report quantities and a fix for "RDL placed nothing".
- Needs AutoCAD 2014 or newer (the 3.3 guide), was 2013.
- "Look inside the user guide": eight pages of the 3.3 guide in guide-v33
  (rendered at 1280 x 720); guide-v32 removed. Pages 28 and 30 shown
  beside "New in 3.3".
- Home spotlight text mentions the single line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018jJ7z3HcJTWCRpFMsrqo1H
</commit_message>
<xml_diff>
--- a/public/roadpro/RoadPro_Shortcuts.xlsx
+++ b/public/roadpro/RoadPro_Shortcuts.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -560,14 +560,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RoadPro v3.2 - Shortcut Keys</t>
+          <t>RoadPro v3.3 - Shortcut Keys</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AutoCAD road builder plugin  |  09-Oct-2026  |  Developed by https://www.exceltokml.com/</t>
+          <t>AutoCAD road builder plugin  |  12-Oct-2026  |  Developed by https://www.exceltokml.com/</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="34" customHeight="1">
+    <row r="11" ht="46" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>RDW</t>
@@ -693,11 +693,11 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Lane widening: extra lane from start to end chainage that comes back, straight or curve taper, fillet or direct link. Both sides can use different chainages and radius</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
+          <t>Lane widening: extra lane from start to end chainage that comes back, straight or curve taper, fillet or direct link. Both sides can use different chainages and radius. Barricades, cones and kerb move to the new edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>RDT</t>
@@ -710,11 +710,11 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Road taper: wider (+) or narrower (-) from any start to any end chainage, new width continues to the road end. Both sides can use different chainages and radius</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
+          <t>Road taper: wider (+) or narrower (-) from any start to any end chainage, new width continues to the road end. Both sides can use different chainages and radius. Barricades, cones and kerb follow the new edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>RDJ</t>
@@ -727,7 +727,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Road junction / tie-in: join a new road with kerb-return radius, opened edge, corner surface, barricades, STOP / GIVE WAY and turning-area markings</t>
+          <t>Road junction / tie-in: join a new road with kerb-return radius, opened edge, corner surface, corner treatment (same as main road, barricades, traffic cones or kerb stone), STOP / GIVE WAY, turning-area markings, auxiliary lane and island</t>
         </is>
       </c>
     </row>
@@ -744,121 +744,145 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Road markings: white edge lines and lane line (broken 3 m / 6 m, solid on bends and junction approaches). Draw again to refresh, or Remove</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+          <t>Road markings: white centre line (L1 / L2 / L2A by speed, or double / single continuous), yellow L4 edge lines, arrows. Draw again to refresh, or Remove</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>RDL</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>ROADLINE</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>NEW in 3.3 - Single line: one run of barricades, traffic cones or kerb stone along any line, polyline, arc, spline, circle or ellipse. On the line, offset left / right or both sides, from / to distance, quantity label</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>ROADPRORESET</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Restore all settings to defaults (no shortcut, on purpose, so you don't reset by accident)</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Useful AutoCAD keys while using RoadPro</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Use</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="C19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Undo the whole road in one step</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="C20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Open the command history to see the summary and the Excel file path</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="C21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Enter</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Finish drawing the centre line, or skip a prompt (such as placing tables)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="C22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Esc</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Cancel the command</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="C23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>APPLOAD</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Load RoadPro.lsp, or add it to the Startup Suite</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n"/>
-    </row>
-    <row r="25" ht="44" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Note: RDR, RDRAD, RDSEC, RDX, RDW, RDT, RDJ and RDM all start by asking you to select the road's centre line (layer ROAD-CL). Turning radius: Match existing (default) or Manual, measured at the centre line. Chainage boxes accept 100 or 0+100. Sign sizes, warning distances and line patterns follow Oman HDS 2017 Sec.19 (check QTCM in Qatar).</t>
+      <c r="C24" s="11" t="n"/>
+    </row>
+    <row r="26" ht="78" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Note: RDR, RDRAD, RDSEC, RDX, RDW, RDT, RDJ and RDM start by asking you to select the road's centre line (layer ROAD-CL). RDL works on any line you select. Edge treatment: barricades, traffic cones or kerb stone. Chainage boxes accept 100 or 0+100. Sign sizes, warning distances and line patterns follow Oman HDS 2017 Sec.19 (check QTCM in Qatar). Full step-by-step manual: RoadPro_User_Guide.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>https://www.exceltokml.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Developed by https://www.exceltokml.com/</t>
         </is>
@@ -866,17 +890,17 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B24:C24"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="A17:C17"/>
     <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="B18:C18"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <hyperlinks>
@@ -886,7 +910,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C&amp;9 RoadPro v3.2  |  Developed by https://www.exceltokml.com/</oddFooter>
+    <oddFooter>&amp;C&amp;9 RoadPro v3.3  |  Developed by https://www.exceltokml.com/</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>